<commit_message>
Added sensitivity to outlier
</commit_message>
<xml_diff>
--- a/pandemic-loss-modeling/exceedance_results/bernstein_1600.xlsx
+++ b/pandemic-loss-modeling/exceedance_results/bernstein_1600.xlsx
@@ -393,7 +393,7 @@
         <v>0.001</v>
       </c>
       <c r="B2">
-        <v>0.9599900153990543</v>
+        <v>0.890268892028197</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -401,7 +401,7 @@
         <v>0.002</v>
       </c>
       <c r="B3">
-        <v>0.9230400330954205</v>
+        <v>0.802195185960294</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -409,7 +409,7 @@
         <v>7.2</v>
       </c>
       <c r="B4">
-        <v>0.00312329197276536</v>
+        <v>0.001093934894911173</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -417,7 +417,7 @@
         <v>28</v>
       </c>
       <c r="B5">
-        <v>0.0007909408080863116</v>
+        <v>0.0002796394860172561</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -425,7 +425,7 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>0.00048924703094509</v>
+        <v>0.0001736068601425977</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -433,7 +433,7 @@
         <v>86</v>
       </c>
       <c r="B7">
-        <v>0.0002538997096630055</v>
+        <v>9.055641475553972E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -441,7 +441,7 @@
         <v>150</v>
       </c>
       <c r="B8">
-        <v>0.0001445274328776631</v>
+        <v>5.177762395711147E-05</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -449,7 +449,7 @@
         <v>200</v>
       </c>
       <c r="B9">
-        <v>0.0001079913333998318</v>
+        <v>3.877820723644303E-05</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -457,7 +457,7 @@
         <v>220</v>
       </c>
       <c r="B10">
-        <v>9.805225465561176E-05</v>
+        <v>3.52363346789119E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -465,7 +465,7 @@
         <v>250</v>
       </c>
       <c r="B11">
-        <v>8.61424332684273E-05</v>
+        <v>3.098839865952652E-05</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -473,7 +473,7 @@
         <v>280</v>
       </c>
       <c r="B12">
-        <v>7.679933369250712E-05</v>
+        <v>2.7652714609963E-05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added 0.01 thresh to gphs
</commit_message>
<xml_diff>
--- a/pandemic-loss-modeling/exceedance_results/bernstein_1600.xlsx
+++ b/pandemic-loss-modeling/exceedance_results/bernstein_1600.xlsx
@@ -377,7 +377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -390,89 +390,81 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="B2">
-        <v>0.890268892028197</v>
+        <v>0.4474311872472255</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>0.002</v>
+        <v>7.2</v>
       </c>
       <c r="B3">
-        <v>0.802195185960294</v>
+        <v>0.001093934894911173</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>7.2</v>
+        <v>28</v>
       </c>
       <c r="B4">
-        <v>0.001093934894911173</v>
+        <v>0.0002796394860172561</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B5">
-        <v>0.0002796394860172561</v>
+        <v>0.0001736068601425977</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="B6">
-        <v>0.0001736068601425977</v>
+        <v>9.055641475553972E-05</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>86</v>
+        <v>150</v>
       </c>
       <c r="B7">
-        <v>9.055641475553972E-05</v>
+        <v>5.177762395711147E-05</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="B8">
-        <v>5.177762395711147E-05</v>
+        <v>3.877820723644303E-05</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="B9">
-        <v>3.877820723644303E-05</v>
+        <v>3.52363346789119E-05</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="B10">
-        <v>3.52363346789119E-05</v>
+        <v>3.098839865952652E-05</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="B11">
-        <v>3.098839865952652E-05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12">
-        <v>280</v>
-      </c>
-      <c r="B12">
         <v>2.7652714609963E-05</v>
       </c>
     </row>

</xml_diff>